<commit_message>
Updated sample sample forms.
</commit_message>
<xml_diff>
--- a/www/sosdar-StatsInExcel-MatchScoreWizzard-EnglishSampleForm.xlsx
+++ b/www/sosdar-StatsInExcel-MatchScoreWizzard-EnglishSampleForm.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5266823fe773b5e1/downloads/MatchScoreWizzard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sos\downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{66E7428E-9AF0-45E1-949E-E000AF96522F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AE3C385-B63C-4DA3-B3E9-DC9E8361A110}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6052A8C8-A93F-4F0B-A854-6B0FC7D7A434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{EBB2CA61-FEA4-4302-A819-98635C214671}"/>
   </bookViews>
   <sheets>
-    <sheet name="FORM" sheetId="3" r:id="rId1"/>
+    <sheet name="FORM" sheetId="4" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="53">
   <si>
     <t>E-Mail</t>
   </si>
@@ -210,6 +210,580 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> key to navigate between cells</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+Welcome to the “MatchScore Wizzard - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2026 World Cup Group Stage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Contest to take place during the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>72 matches</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> of the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Groups Stage of the 2026 World Cup</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">. Contest details are described below.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>1.  Enrollment</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Enrollment is completely free and will be managed electronically (there is NO need to print out forms). Complete all form fields using Microsoft Excel. Fill in: full name or nickname (for example, "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Lio Messi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>" or "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Best of the World</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">"), e-mail, and your predictions for every match. Then, press </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>F12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to save your form as, for example, "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Lionel Messi.xlsx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">" or "Best of the world.xlsx". Send your form to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>AdminEmail@domain</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (one xlsx file for each form) before the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>World Cup</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> kick-off on </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>June 11</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <vertAlign val="superscript"/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>th</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2.  Scoring system</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+For each match you may get between zero (0) and three (3) points according to the following rules:
+■ Three (3) points if your prediction exactly matches the official final score.
+■ Two (2) points if you correctly guess a winner team and the goals scored by either team, but not both.
+■ One (1) point if you correctly predict a tied match, but you failed to correctly predict the exact number of goals scored.
+■ Zero (0) points if you fail to predict a winner team or a tied match.
+Example:  The official result of the match A vs B es </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2-0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> in favor of A.
+If your prediction was </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> in favor of team A, you will get three points.
+If your prediction was </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-1, 1-</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>, 3-</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>, 4-</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>, 5-</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, ...,  in favor of team A, you will get two points because you predicted A winning the match and you correctly guessed the goals scored by one of the two teams.
+If your prediction was 3-1, 4-1, 5-1,..., 3-2, 4-2, 5-2,... or any other score in favor of  A, you will get one point because you predicted the winner (team A) without guessing correctly the goals scored by neither team.  
+If your prediction was B winning or a tie, you will get zero points.
+Your final score will be the total number of points across all </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>72</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> matches.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>3. License and use</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+This Excel form is provided for personal and non-commercial use only as part of an entertainment activity. You may use and adapt it for friendly prediction contests. Commercial use, resale, or redistribution as your own product is not permitted.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>4. Copyright</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+© MatchScore Wizzard. All rights reserved._x000B_The layout, structure, wording, and presentation of this file are protected by copyright law.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>5. Entertainment-only disclaimer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+This contest and its scoring system are intended solely for entertainment purposes. No gambling, betting, prizes, or financial rewards are involved.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>6. Independent contests and affiliations</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Each contest using this form is independently organized by its administrator._x000B_MatchScore Wizzard does not manage contests and is not affiliated with organizers, participants, or any sporting authority.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>❤️</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Optional Support</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+If you enjoy using MatchScore Wizzard and wish to support its continued development, voluntary, non-tax-deductible contributions are appreciated. Support is optional and does not affect participation, scoring, or results.
+(You may go to https://paypal.me/blessingSOSDAR, use the PayPal account </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="8"/>
+        <color rgb="FF1F78B4"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>polluelo02@hotmail.com,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1" tint="0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> or scan or click the QR code shown below.)
+</t>
     </r>
   </si>
 </sst>
@@ -220,16 +794,10 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d;@"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
@@ -280,6 +848,50 @@
       <u/>
       <sz val="10"/>
       <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1" tint="0.249977111117893"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1" tint="0.249977111117893"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <vertAlign val="superscript"/>
+      <sz val="8"/>
+      <color theme="1" tint="0.249977111117893"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="8"/>
+      <color theme="1" tint="0.249977111117893"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="8"/>
+      <color rgb="FF1F78B4"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -361,13 +973,19 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -375,72 +993,72 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -451,9 +1069,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF1F78B4"/>
       <color rgb="FFA6CEE3"/>
       <color rgb="FFFC8D62"/>
-      <color rgb="FF1F78B4"/>
       <color rgb="FFFF7F00"/>
       <color rgb="FFE5C494"/>
       <color rgb="FFFDBF6F"/>
@@ -472,1425 +1090,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="absolute">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>22654</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>781</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>819288</xdr:colOff>
-      <xdr:row>79</xdr:row>
-      <xdr:rowOff>36634</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1027" name="Text Box 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B8A14F2B-36C3-04BA-5266-7E6BB5576CED}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="22654" y="372012"/>
-          <a:ext cx="3119269" cy="11802891"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="9"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="t" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Welcome to the “</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>MatchScore Wizzard - 2026 World Cup Group Stage Contest</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> to take place during the </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>72 matches of the group stage of the 2026 World Cup</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>. Contest details are described below.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>1.  Enrollment</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Enrollment is completely free and will be managed electronically (there is </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>NO</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> need to print out your form). Complete your form using Microsoft Excel. Fill in: full name or nickname (for example, "Lio Messi" or "Best of the World"), e-mail, and your predictions for every match. Then, press </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>F12</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> to save your form as, for example, "</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Lionel Messi.xlsx</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>" or "</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Best of the world.xlsx</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>". Send your form(s) to </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>AdminEmail@domain </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>(one xlsx file for each form) before the </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>World Cup</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> kick-off on </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>June 11</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="30000">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>th</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>2.  Scoring system</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>For each match you may get between zero (0) and three (3) points according to the following rules:</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>■ Three </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>(3)</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> points if your prediction exactly matches the official final score.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>■ Two </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>(2)</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> points if you correctly guess a winner team and the goals scored by either team, but not both.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>■ One </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>(1)</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> point if you correctly predict a tied match, but you failed to correctly predict the exact number of goals scored.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>■ Zero </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>(0)</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> points if you fail to predict a winner team or a tied match.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="sng" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Example:</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>  The official result of the match A vs B</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>es </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>2-0</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> in favor of A.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>If your prediction was </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="sng" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>2</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>-</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="sng" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>0</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> in favor of team </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>A</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>, you will get three points.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>If your prediction was </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="sng" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>2</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>-1, 1-</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="sng" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>0</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>, 3-</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="sng" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>0</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>, 4-</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="sng" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>0</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>, 5-</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="sng" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>0</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>, ...,  in favor of team </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>A</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>, you will get </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>two points</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> because you predicted </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>A</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> winning the match and you correctly guessed the goals scored by one of the two teams.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>If your prediction was 3-1, 4-1, 5-1,..., 3-2, 4-2, 5-2,... or any other score in favor of  </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>A</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>, you will get </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>one point</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> because you predicted the winner (team </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>A</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>) without guessing correctly the goals scored by neither team.  </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>If your prediction was </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>B</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> winning or a tie, you will get </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>zero points</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Your final score will be the total number of points across all </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>72</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> matches.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>3. License and use</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>This Excel form is provided for </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>personal and non-commercial use only</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> as part of an entertainment activity. You may use and adapt it for friendly prediction contests. Commercial use, resale, or redistribution as your own product is not permitted.</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>4. Copyright</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>© MatchScore Wizzard. All rights reserved.</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>The layout, structure, wording, and presentation of this file are protected by copyright law.</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="just" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>5. Entertainment-only disclaimer</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>This contest and its scoring system are intended </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>solely for entertainment purposes</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>. No gambling, betting, prizes, or financial rewards are involved.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>6.</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1" baseline="0">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> Independent contests and affiliations</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="800" b="1">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Each contest using this form is independently organized by its administrator.</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>MatchScore Wizzard does not manage contests and is not affiliated with organizers, participants, or any sporting authority.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>❤️ Optional Support</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>If you enjoy using MatchScore Wizzard and wish to support its continued development, </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>voluntary, non-tax-deductible contributions</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> are appreciated. Support is optional and </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" b="1">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>does not affect participation, scoring, or results</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>(You may use the </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:effectLst/>
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>PayPal</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>polluelo02@hotmail.com account or its QR code shown below.)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:endParaRPr lang="en-US" sz="800" b="1">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -1906,10 +1105,10 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="1026" name="Text Box 2">
+        <xdr:cNvPr id="3" name="Text Box 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{78E488B4-6263-E538-43BA-256F6BD00DC2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6B217DA-022C-4749-BC58-0CFD8C5B42B2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1919,8 +1118,8 @@
       </xdr:nvSpPr>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="0" y="9404350"/>
-          <a:ext cx="0" cy="8788400"/>
+          <a:off x="0" y="12204700"/>
+          <a:ext cx="0" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2397,10 +1596,11 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{48B3DE83-8ED5-3952-3116-7A4B14647DCC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F2B6CE36-3447-4F48-B646-A1813765B4E4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2409,7 +1609,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -2423,8 +1623,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="724161" y="9283846"/>
-          <a:ext cx="1602274" cy="1599574"/>
+          <a:off x="723422" y="9292110"/>
+          <a:ext cx="1602404" cy="1601139"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2817,7 +2017,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A29A7B56-6BD6-4BFE-9B6D-2424CEA35A53}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4794D882-0076-4D28-9C89-2D7ECD9E5301}">
   <dimension ref="A1:L79"/>
   <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="11.75" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -2836,44 +2036,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
     </row>
     <row r="2" spans="1:12" ht="12" x14ac:dyDescent="0.6">
-      <c r="F2" s="21" t="s">
+      <c r="A2" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="26"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
       <c r="F3" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="22"/>
-      <c r="H3" s="23"/>
-      <c r="I3" s="23"/>
-      <c r="J3" s="23"/>
-      <c r="K3" s="23"/>
-      <c r="L3" s="24"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="20"/>
     </row>
     <row r="4" spans="1:12" ht="3.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="26"/>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -2883,17 +2100,27 @@
       <c r="L4" s="4"/>
     </row>
     <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="26"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="26"/>
       <c r="F5" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="G5" s="18"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="20"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="23"/>
     </row>
     <row r="6" spans="1:12" ht="3.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="26"/>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
       <c r="F6" s="3"/>
       <c r="G6" s="4"/>
       <c r="H6" s="2"/>
@@ -2903,21 +2130,31 @@
       <c r="L6" s="4"/>
     </row>
     <row r="7" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="26"/>
+      <c r="B7" s="26"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
       <c r="F7" s="5" t="s">
         <v>24</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H7" s="16" t="s">
+      <c r="H7" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="16"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
     </row>
     <row r="8" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="26"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
       <c r="F8" s="3">
         <v>1</v>
       </c>
@@ -2937,6 +2174,11 @@
       <c r="L8" s="7"/>
     </row>
     <row r="9" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="26"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
       <c r="F9" s="3">
         <v>2</v>
       </c>
@@ -2954,6 +2196,11 @@
       <c r="L9" s="7"/>
     </row>
     <row r="10" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="26"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="26"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
       <c r="F10" s="3">
         <v>3</v>
       </c>
@@ -2973,6 +2220,11 @@
       <c r="L10" s="7"/>
     </row>
     <row r="11" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="26"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
       <c r="F11" s="3">
         <v>4</v>
       </c>
@@ -2990,6 +2242,11 @@
       <c r="L11" s="7"/>
     </row>
     <row r="12" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="26"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
       <c r="F12" s="3">
         <v>5</v>
       </c>
@@ -3009,6 +2266,11 @@
       <c r="L12" s="7"/>
     </row>
     <row r="13" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="26"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
       <c r="F13" s="3">
         <v>6</v>
       </c>
@@ -3026,6 +2288,11 @@
       <c r="L13" s="7"/>
     </row>
     <row r="14" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="26"/>
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
       <c r="F14" s="3">
         <v>7</v>
       </c>
@@ -3043,6 +2310,11 @@
       <c r="L14" s="7"/>
     </row>
     <row r="15" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="26"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
       <c r="F15" s="3">
         <v>8</v>
       </c>
@@ -3060,6 +2332,11 @@
       <c r="L15" s="7"/>
     </row>
     <row r="16" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="26"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
       <c r="F16" s="3">
         <v>9</v>
       </c>
@@ -3078,7 +2355,12 @@
       </c>
       <c r="L16" s="7"/>
     </row>
-    <row r="17" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="26"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
       <c r="F17" s="3">
         <v>10</v>
       </c>
@@ -3095,7 +2377,12 @@
       </c>
       <c r="L17" s="7"/>
     </row>
-    <row r="18" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="26"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
       <c r="F18" s="3">
         <v>11</v>
       </c>
@@ -3112,7 +2399,12 @@
       </c>
       <c r="L18" s="7"/>
     </row>
-    <row r="19" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="26"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
       <c r="F19" s="3">
         <v>12</v>
       </c>
@@ -3129,7 +2421,12 @@
       </c>
       <c r="L19" s="7"/>
     </row>
-    <row r="20" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="26"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
       <c r="F20" s="3">
         <v>13</v>
       </c>
@@ -3148,7 +2445,12 @@
       </c>
       <c r="L20" s="7"/>
     </row>
-    <row r="21" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="26"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
       <c r="F21" s="3">
         <v>14</v>
       </c>
@@ -3165,7 +2467,12 @@
       </c>
       <c r="L21" s="7"/>
     </row>
-    <row r="22" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A22" s="26"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="3">
         <v>15</v>
       </c>
@@ -3182,7 +2489,12 @@
       </c>
       <c r="L22" s="7"/>
     </row>
-    <row r="23" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23" s="26"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
       <c r="F23" s="3">
         <v>16</v>
       </c>
@@ -3199,7 +2511,12 @@
       </c>
       <c r="L23" s="7"/>
     </row>
-    <row r="24" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A24" s="26"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
       <c r="F24" s="3">
         <v>17</v>
       </c>
@@ -3218,7 +2535,12 @@
       </c>
       <c r="L24" s="7"/>
     </row>
-    <row r="25" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A25" s="26"/>
+      <c r="B25" s="26"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
       <c r="F25" s="3">
         <v>18</v>
       </c>
@@ -3235,7 +2557,12 @@
       </c>
       <c r="L25" s="7"/>
     </row>
-    <row r="26" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A26" s="26"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
       <c r="F26" s="3">
         <v>19</v>
       </c>
@@ -3252,7 +2579,12 @@
       </c>
       <c r="L26" s="7"/>
     </row>
-    <row r="27" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A27" s="26"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
       <c r="F27" s="3">
         <v>20</v>
       </c>
@@ -3269,7 +2601,12 @@
       </c>
       <c r="L27" s="7"/>
     </row>
-    <row r="28" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A28" s="26"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
       <c r="F28" s="3">
         <v>21</v>
       </c>
@@ -3288,7 +2625,12 @@
       </c>
       <c r="L28" s="7"/>
     </row>
-    <row r="29" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A29" s="26"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
       <c r="F29" s="3">
         <v>22</v>
       </c>
@@ -3305,7 +2647,12 @@
       </c>
       <c r="L29" s="7"/>
     </row>
-    <row r="30" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30" s="26"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
       <c r="F30" s="3">
         <v>23</v>
       </c>
@@ -3322,7 +2669,12 @@
       </c>
       <c r="L30" s="7"/>
     </row>
-    <row r="31" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A31" s="26"/>
+      <c r="B31" s="26"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
       <c r="F31" s="3">
         <v>24</v>
       </c>
@@ -3339,7 +2691,12 @@
       </c>
       <c r="L31" s="7"/>
     </row>
-    <row r="32" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A32" s="26"/>
+      <c r="B32" s="26"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
       <c r="F32" s="3">
         <v>25</v>
       </c>
@@ -3358,7 +2715,12 @@
       </c>
       <c r="L32" s="7"/>
     </row>
-    <row r="33" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33" s="26"/>
+      <c r="B33" s="26"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="26"/>
       <c r="F33" s="3">
         <v>26</v>
       </c>
@@ -3375,7 +2737,12 @@
       </c>
       <c r="L33" s="7"/>
     </row>
-    <row r="34" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A34" s="26"/>
+      <c r="B34" s="26"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="26"/>
       <c r="F34" s="3">
         <v>27</v>
       </c>
@@ -3392,7 +2759,12 @@
       </c>
       <c r="L34" s="7"/>
     </row>
-    <row r="35" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A35" s="26"/>
+      <c r="B35" s="26"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
       <c r="F35" s="3">
         <v>28</v>
       </c>
@@ -3409,7 +2781,12 @@
       </c>
       <c r="L35" s="7"/>
     </row>
-    <row r="36" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36" s="26"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="26"/>
       <c r="F36" s="3">
         <v>29</v>
       </c>
@@ -3428,7 +2805,12 @@
       </c>
       <c r="L36" s="7"/>
     </row>
-    <row r="37" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A37" s="26"/>
+      <c r="B37" s="26"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="26"/>
       <c r="F37" s="3">
         <v>30</v>
       </c>
@@ -3445,7 +2827,12 @@
       </c>
       <c r="L37" s="7"/>
     </row>
-    <row r="38" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A38" s="26"/>
+      <c r="B38" s="26"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="26"/>
       <c r="F38" s="3">
         <v>31</v>
       </c>
@@ -3462,7 +2849,12 @@
       </c>
       <c r="L38" s="7"/>
     </row>
-    <row r="39" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A39" s="26"/>
+      <c r="B39" s="26"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="26"/>
       <c r="F39" s="3">
         <v>32</v>
       </c>
@@ -3479,7 +2871,12 @@
       </c>
       <c r="L39" s="7"/>
     </row>
-    <row r="40" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A40" s="26"/>
+      <c r="B40" s="26"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
       <c r="F40" s="3">
         <v>33</v>
       </c>
@@ -3498,7 +2895,12 @@
       </c>
       <c r="L40" s="7"/>
     </row>
-    <row r="41" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A41" s="26"/>
+      <c r="B41" s="26"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="26"/>
+      <c r="E41" s="26"/>
       <c r="F41" s="3">
         <v>34</v>
       </c>
@@ -3515,7 +2917,12 @@
       </c>
       <c r="L41" s="7"/>
     </row>
-    <row r="42" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A42" s="26"/>
+      <c r="B42" s="26"/>
+      <c r="C42" s="26"/>
+      <c r="D42" s="26"/>
+      <c r="E42" s="26"/>
       <c r="F42" s="3">
         <v>35</v>
       </c>
@@ -3532,7 +2939,12 @@
       </c>
       <c r="L42" s="7"/>
     </row>
-    <row r="43" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A43" s="26"/>
+      <c r="B43" s="26"/>
+      <c r="C43" s="26"/>
+      <c r="D43" s="26"/>
+      <c r="E43" s="26"/>
       <c r="F43" s="3">
         <v>36</v>
       </c>
@@ -3549,7 +2961,12 @@
       </c>
       <c r="L43" s="7"/>
     </row>
-    <row r="44" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A44" s="26"/>
+      <c r="B44" s="26"/>
+      <c r="C44" s="26"/>
+      <c r="D44" s="26"/>
+      <c r="E44" s="26"/>
       <c r="F44" s="3">
         <v>37</v>
       </c>
@@ -3568,7 +2985,12 @@
       </c>
       <c r="L44" s="7"/>
     </row>
-    <row r="45" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A45" s="26"/>
+      <c r="B45" s="26"/>
+      <c r="C45" s="26"/>
+      <c r="D45" s="26"/>
+      <c r="E45" s="26"/>
       <c r="F45" s="3">
         <v>38</v>
       </c>
@@ -3585,7 +3007,12 @@
       </c>
       <c r="L45" s="7"/>
     </row>
-    <row r="46" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A46" s="26"/>
+      <c r="B46" s="26"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="26"/>
+      <c r="E46" s="26"/>
       <c r="F46" s="3">
         <v>39</v>
       </c>
@@ -3602,7 +3029,12 @@
       </c>
       <c r="L46" s="7"/>
     </row>
-    <row r="47" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A47" s="26"/>
+      <c r="B47" s="26"/>
+      <c r="C47" s="26"/>
+      <c r="D47" s="26"/>
+      <c r="E47" s="26"/>
       <c r="F47" s="3">
         <v>40</v>
       </c>
@@ -3619,7 +3051,12 @@
       </c>
       <c r="L47" s="7"/>
     </row>
-    <row r="48" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A48" s="26"/>
+      <c r="B48" s="26"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="26"/>
+      <c r="E48" s="26"/>
       <c r="F48" s="3">
         <v>41</v>
       </c>
@@ -3638,7 +3075,12 @@
       </c>
       <c r="L48" s="7"/>
     </row>
-    <row r="49" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A49" s="26"/>
+      <c r="B49" s="26"/>
+      <c r="C49" s="26"/>
+      <c r="D49" s="26"/>
+      <c r="E49" s="26"/>
       <c r="F49" s="3">
         <v>42</v>
       </c>
@@ -3655,7 +3097,12 @@
       </c>
       <c r="L49" s="7"/>
     </row>
-    <row r="50" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A50" s="26"/>
+      <c r="B50" s="26"/>
+      <c r="C50" s="26"/>
+      <c r="D50" s="26"/>
+      <c r="E50" s="26"/>
       <c r="F50" s="3">
         <v>43</v>
       </c>
@@ -3672,7 +3119,12 @@
       </c>
       <c r="L50" s="7"/>
     </row>
-    <row r="51" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A51" s="26"/>
+      <c r="B51" s="26"/>
+      <c r="C51" s="26"/>
+      <c r="D51" s="26"/>
+      <c r="E51" s="26"/>
       <c r="F51" s="3">
         <v>44</v>
       </c>
@@ -3689,7 +3141,12 @@
       </c>
       <c r="L51" s="7"/>
     </row>
-    <row r="52" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A52" s="26"/>
+      <c r="B52" s="26"/>
+      <c r="C52" s="26"/>
+      <c r="D52" s="26"/>
+      <c r="E52" s="26"/>
       <c r="F52" s="3">
         <v>45</v>
       </c>
@@ -3708,7 +3165,12 @@
       </c>
       <c r="L52" s="7"/>
     </row>
-    <row r="53" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A53" s="26"/>
+      <c r="B53" s="26"/>
+      <c r="C53" s="26"/>
+      <c r="D53" s="26"/>
+      <c r="E53" s="26"/>
       <c r="F53" s="3">
         <v>46</v>
       </c>
@@ -3725,7 +3187,12 @@
       </c>
       <c r="L53" s="7"/>
     </row>
-    <row r="54" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A54" s="26"/>
+      <c r="B54" s="26"/>
+      <c r="C54" s="26"/>
+      <c r="D54" s="26"/>
+      <c r="E54" s="26"/>
       <c r="F54" s="3">
         <v>47</v>
       </c>
@@ -3742,7 +3209,12 @@
       </c>
       <c r="L54" s="7"/>
     </row>
-    <row r="55" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A55" s="26"/>
+      <c r="B55" s="26"/>
+      <c r="C55" s="26"/>
+      <c r="D55" s="26"/>
+      <c r="E55" s="26"/>
       <c r="F55" s="3">
         <v>48</v>
       </c>
@@ -3759,7 +3231,12 @@
       </c>
       <c r="L55" s="7"/>
     </row>
-    <row r="56" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A56" s="26"/>
+      <c r="B56" s="26"/>
+      <c r="C56" s="26"/>
+      <c r="D56" s="26"/>
+      <c r="E56" s="26"/>
       <c r="F56" s="3">
         <v>49</v>
       </c>
@@ -3778,7 +3255,12 @@
       </c>
       <c r="L56" s="7"/>
     </row>
-    <row r="57" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A57" s="26"/>
+      <c r="B57" s="26"/>
+      <c r="C57" s="26"/>
+      <c r="D57" s="26"/>
+      <c r="E57" s="26"/>
       <c r="F57" s="3">
         <v>50</v>
       </c>
@@ -3795,7 +3277,12 @@
       </c>
       <c r="L57" s="7"/>
     </row>
-    <row r="58" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A58" s="26"/>
+      <c r="B58" s="26"/>
+      <c r="C58" s="26"/>
+      <c r="D58" s="26"/>
+      <c r="E58" s="26"/>
       <c r="F58" s="3">
         <v>51</v>
       </c>
@@ -3812,7 +3299,12 @@
       </c>
       <c r="L58" s="7"/>
     </row>
-    <row r="59" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A59" s="26"/>
+      <c r="B59" s="26"/>
+      <c r="C59" s="26"/>
+      <c r="D59" s="26"/>
+      <c r="E59" s="26"/>
       <c r="F59" s="3">
         <v>52</v>
       </c>
@@ -3829,7 +3321,12 @@
       </c>
       <c r="L59" s="7"/>
     </row>
-    <row r="60" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A60" s="26"/>
+      <c r="B60" s="26"/>
+      <c r="C60" s="26"/>
+      <c r="D60" s="26"/>
+      <c r="E60" s="26"/>
       <c r="F60" s="3">
         <v>53</v>
       </c>
@@ -3846,7 +3343,12 @@
       </c>
       <c r="L60" s="7"/>
     </row>
-    <row r="61" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A61" s="26"/>
+      <c r="B61" s="26"/>
+      <c r="C61" s="26"/>
+      <c r="D61" s="26"/>
+      <c r="E61" s="26"/>
       <c r="F61" s="3">
         <v>54</v>
       </c>
@@ -3863,7 +3365,12 @@
       </c>
       <c r="L61" s="7"/>
     </row>
-    <row r="62" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A62" s="26"/>
+      <c r="B62" s="26"/>
+      <c r="C62" s="26"/>
+      <c r="D62" s="26"/>
+      <c r="E62" s="26"/>
       <c r="F62" s="3">
         <v>55</v>
       </c>
@@ -3882,7 +3389,12 @@
       </c>
       <c r="L62" s="7"/>
     </row>
-    <row r="63" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A63" s="26"/>
+      <c r="B63" s="26"/>
+      <c r="C63" s="26"/>
+      <c r="D63" s="26"/>
+      <c r="E63" s="26"/>
       <c r="F63" s="3">
         <v>56</v>
       </c>
@@ -3899,7 +3411,12 @@
       </c>
       <c r="L63" s="7"/>
     </row>
-    <row r="64" spans="6:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A64" s="26"/>
+      <c r="B64" s="26"/>
+      <c r="C64" s="26"/>
+      <c r="D64" s="26"/>
+      <c r="E64" s="26"/>
       <c r="F64" s="3">
         <v>57</v>
       </c>
@@ -3916,8 +3433,12 @@
       </c>
       <c r="L64" s="7"/>
     </row>
-    <row r="65" spans="4:12" ht="13" x14ac:dyDescent="0.6">
-      <c r="D65"/>
+    <row r="65" spans="1:12" ht="13" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A65" s="26"/>
+      <c r="B65" s="26"/>
+      <c r="C65" s="26"/>
+      <c r="D65" s="26"/>
+      <c r="E65" s="26"/>
       <c r="F65" s="3">
         <v>58</v>
       </c>
@@ -3934,7 +3455,12 @@
       </c>
       <c r="L65" s="7"/>
     </row>
-    <row r="66" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A66" s="26"/>
+      <c r="B66" s="26"/>
+      <c r="C66" s="26"/>
+      <c r="D66" s="26"/>
+      <c r="E66" s="26"/>
       <c r="F66" s="3">
         <v>59</v>
       </c>
@@ -3951,7 +3477,12 @@
       </c>
       <c r="L66" s="7"/>
     </row>
-    <row r="67" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A67" s="26"/>
+      <c r="B67" s="26"/>
+      <c r="C67" s="26"/>
+      <c r="D67" s="26"/>
+      <c r="E67" s="26"/>
       <c r="F67" s="3">
         <v>60</v>
       </c>
@@ -3968,7 +3499,12 @@
       </c>
       <c r="L67" s="7"/>
     </row>
-    <row r="68" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A68" s="26"/>
+      <c r="B68" s="26"/>
+      <c r="C68" s="26"/>
+      <c r="D68" s="26"/>
+      <c r="E68" s="26"/>
       <c r="F68" s="3">
         <v>61</v>
       </c>
@@ -3987,7 +3523,12 @@
       </c>
       <c r="L68" s="7"/>
     </row>
-    <row r="69" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A69" s="26"/>
+      <c r="B69" s="26"/>
+      <c r="C69" s="26"/>
+      <c r="D69" s="26"/>
+      <c r="E69" s="26"/>
       <c r="F69" s="3">
         <v>62</v>
       </c>
@@ -4004,7 +3545,12 @@
       </c>
       <c r="L69" s="7"/>
     </row>
-    <row r="70" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A70" s="26"/>
+      <c r="B70" s="26"/>
+      <c r="C70" s="26"/>
+      <c r="D70" s="26"/>
+      <c r="E70" s="26"/>
       <c r="F70" s="3">
         <v>63</v>
       </c>
@@ -4021,7 +3567,12 @@
       </c>
       <c r="L70" s="7"/>
     </row>
-    <row r="71" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A71" s="26"/>
+      <c r="B71" s="26"/>
+      <c r="C71" s="26"/>
+      <c r="D71" s="26"/>
+      <c r="E71" s="26"/>
       <c r="F71" s="3">
         <v>64</v>
       </c>
@@ -4038,7 +3589,12 @@
       </c>
       <c r="L71" s="7"/>
     </row>
-    <row r="72" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A72" s="26"/>
+      <c r="B72" s="26"/>
+      <c r="C72" s="26"/>
+      <c r="D72" s="26"/>
+      <c r="E72" s="26"/>
       <c r="F72" s="3">
         <v>65</v>
       </c>
@@ -4055,7 +3611,12 @@
       </c>
       <c r="L72" s="7"/>
     </row>
-    <row r="73" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A73" s="26"/>
+      <c r="B73" s="26"/>
+      <c r="C73" s="26"/>
+      <c r="D73" s="26"/>
+      <c r="E73" s="26"/>
       <c r="F73" s="3">
         <v>66</v>
       </c>
@@ -4072,7 +3633,12 @@
       </c>
       <c r="L73" s="7"/>
     </row>
-    <row r="74" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A74" s="26"/>
+      <c r="B74" s="26"/>
+      <c r="C74" s="26"/>
+      <c r="D74" s="26"/>
+      <c r="E74" s="26"/>
       <c r="F74" s="3">
         <v>67</v>
       </c>
@@ -4091,7 +3657,12 @@
       </c>
       <c r="L74" s="7"/>
     </row>
-    <row r="75" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A75" s="26"/>
+      <c r="B75" s="26"/>
+      <c r="C75" s="26"/>
+      <c r="D75" s="26"/>
+      <c r="E75" s="26"/>
       <c r="F75" s="3">
         <v>68</v>
       </c>
@@ -4108,7 +3679,12 @@
       </c>
       <c r="L75" s="7"/>
     </row>
-    <row r="76" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A76" s="26"/>
+      <c r="B76" s="26"/>
+      <c r="C76" s="26"/>
+      <c r="D76" s="26"/>
+      <c r="E76" s="26"/>
       <c r="F76" s="3">
         <v>69</v>
       </c>
@@ -4125,7 +3701,12 @@
       </c>
       <c r="L76" s="7"/>
     </row>
-    <row r="77" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A77" s="26"/>
+      <c r="B77" s="26"/>
+      <c r="C77" s="26"/>
+      <c r="D77" s="26"/>
+      <c r="E77" s="26"/>
       <c r="F77" s="3">
         <v>70</v>
       </c>
@@ -4142,7 +3723,12 @@
       </c>
       <c r="L77" s="7"/>
     </row>
-    <row r="78" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A78" s="26"/>
+      <c r="B78" s="26"/>
+      <c r="C78" s="26"/>
+      <c r="D78" s="26"/>
+      <c r="E78" s="26"/>
       <c r="F78" s="3">
         <v>71</v>
       </c>
@@ -4159,7 +3745,12 @@
       </c>
       <c r="L78" s="7"/>
     </row>
-    <row r="79" spans="4:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+    <row r="79" spans="1:12" ht="12" x14ac:dyDescent="0.55000000000000004">
+      <c r="A79" s="26"/>
+      <c r="B79" s="26"/>
+      <c r="C79" s="26"/>
+      <c r="D79" s="26"/>
+      <c r="E79" s="26"/>
       <c r="F79" s="3">
         <v>72</v>
       </c>
@@ -4178,19 +3769,16 @@
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" selectLockedCells="1"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="F8:L79">
-    <sortCondition ref="F8:F79"/>
-  </sortState>
-  <mergeCells count="5">
-    <mergeCell ref="H7:L7"/>
+  <mergeCells count="6">
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="G5:L5"/>
     <mergeCell ref="F2:L2"/>
     <mergeCell ref="G3:L3"/>
+    <mergeCell ref="G5:L5"/>
+    <mergeCell ref="H7:L7"/>
+    <mergeCell ref="A2:E79"/>
   </mergeCells>
-  <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="whole" errorStyle="information" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Numeric entry" error="Please enter a whole number greater or equal to 0. Pres ESC to Cancel.a_x000a_nd re-try. _x000a_Thanks." sqref="I8:I79 L8:L79" xr:uid="{EB89CE4D-1741-47A3-811F-22E0FA8FD430}">
+    <dataValidation type="whole" errorStyle="information" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Numeric entry" error="Please enter a whole number greater or equal to 0. Pres ESC to Cancel.a_x000a_nd re-try. _x000a_Thanks." sqref="I8:I79 L8:L79" xr:uid="{ED9ADB03-6726-458D-A03C-536C4AC69775}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>